<commit_message>
ajsute de datos y tablas en diccionario de datos
</commit_message>
<xml_diff>
--- a/Database/diccionario datos-v2.xlsx
+++ b/Database/diccionario datos-v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6fd9368643786761/Documentación actual para corrección - copia/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Documents\trabajo isseg\SGSPCSI\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CD0DC55-1632-4F58-898E-B5C4B745801D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C04C765-FB18-4DFF-9BB5-194BDA85A25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Historial de versiones" sheetId="34" r:id="rId1"/>
@@ -49,6 +49,9 @@
     <sheet name="evento_calendario" sheetId="32" r:id="rId34"/>
     <sheet name="evento_participante" sheetId="33" r:id="rId35"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">INDICE!$A$2:$D$35</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -67,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1711" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="580">
   <si>
     <t>Descripción</t>
   </si>
@@ -1777,6 +1780,45 @@
   </si>
   <si>
     <t>Registra la asignación de usuarios a sistemas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diccionario de datos </t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha y hora en que terminó la vigencia de la asignación. Si está vacía, la relación se considera vigente.	</t>
+  </si>
+  <si>
+    <t>tarea_desarrollo_asignacion_id</t>
+  </si>
+  <si>
+    <t>Identity</t>
+  </si>
+  <si>
+    <t>Identificador único de cada asignación. Se genera automáticamente por el sistema y permite distinguir de forma inequívoca cada relación entre una tarea y un usuario.</t>
+  </si>
+  <si>
+    <t>Identificador de la tarea de desarrollo a la que pertenece la asignación. Vincula el registro con la tarea operativa concreta que se está ejecutando.</t>
+  </si>
+  <si>
+    <t>Identificador del usuario asignado a la tarea. Permite saber qué persona participa en la ejecución del trabajo técnico.</t>
+  </si>
+  <si>
+    <t>rol_tecnico</t>
+  </si>
+  <si>
+    <t>Rol que desempeña el usuario dentro de la tarea. Define su función operativa, por ejemplo RESPONSABLE o PARTICIPANTE.</t>
+  </si>
+  <si>
+    <t>Indica si la asignación está vigente. Valor 1 significa que la persona sigue asignada; valor 0 significa que la asignación ya fue cerrada o desactivada.</t>
+  </si>
+  <si>
+    <t>Fecha y hora en que se creó la asignación. Sirve para trazabilidad, auditoría y control histórico de la participación del usuario en la tarea.</t>
+  </si>
+  <si>
+    <t>Fecha y hora en que terminó la asignación. Si está vacía, la relación sigue vigente. Permite conservar el historial de asignaciones cerradas.</t>
   </si>
 </sst>
 </file>
@@ -1855,7 +1897,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1980,12 +2022,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2080,9 +2131,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4686,19 +4742,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:I35"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="64.85546875" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" customWidth="1"/>
     <col min="4" max="4" width="34.85546875" customWidth="1"/>
-    <col min="8" max="9" width="9" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" customWidth="1"/>
     <col min="10" max="10" width="8.85546875" customWidth="1"/>
     <col min="11" max="11" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="42" t="s">
+        <v>567</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>322</v>
       </c>
@@ -4712,536 +4783,550 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C3" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D3&amp;"'!B4:B55")),0)</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C4" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D4&amp;"'!B4:B55")),0)</f>
         <v>8</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C5" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D5&amp;"'!B4:B55")),0)</f>
         <v>5</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="C6" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D6&amp;"'!B4:B55")),0)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C7" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D7&amp;"'!B4:B55")),0)</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="C8" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D8&amp;"'!B4:B55")),0)</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="C9" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D9&amp;"'!B4:B55")),0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="C10" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D10&amp;"'!B4:B55")),0)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C11" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D11&amp;"'!B4:B55")),0)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D11" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
-        <v>21</v>
-      </c>
       <c r="B12" s="13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C12" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D12&amp;"'!B4:B55")),0)</f>
         <v>5</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="C13" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D13&amp;"'!B4:B55")),0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="C14" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D14&amp;"'!B4:B55")),0)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="32" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>552</v>
+        <v>53</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="C15" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D15&amp;"'!B4:B55")),0)</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>553</v>
+        <v>3</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C16" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D16&amp;"'!B4:B55")),0)</f>
         <v>6</v>
       </c>
       <c r="D16" s="32" t="s">
-        <v>553</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>554</v>
+        <v>37</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C17" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D17&amp;"'!B4:B55")),0)</f>
         <v>6</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>554</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>555</v>
+        <v>13</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C18" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D18&amp;"'!B4:B55")),0)</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>555</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>32</v>
+        <v>551</v>
+      </c>
+      <c r="B19" s="40" t="s">
+        <v>566</v>
       </c>
       <c r="C19" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D19&amp;"'!B4:B55")),0)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>31</v>
+        <v>551</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C20" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D20&amp;"'!B4:B55")),0)</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>35</v>
+        <v>555</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C21" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D21&amp;"'!B4:B55")),0)</f>
         <v>8</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>35</v>
+        <v>555</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>37</v>
+        <v>553</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C22" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D22&amp;"'!B4:B55")),0)</f>
         <v>6</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>37</v>
+        <v>553</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>39</v>
+        <v>554</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C23" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D23&amp;"'!B4:B55")),0)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>39</v>
+        <v>554</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="C24" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D24&amp;"'!B4:B55")),0)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>43</v>
+        <v>552</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="C25" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D25&amp;"'!B4:B55")),0)</f>
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D25" s="32" t="s">
-        <v>43</v>
+        <v>552</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C26" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D26&amp;"'!B4:B55")),0)</f>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D26" s="32" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C27" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D27&amp;"'!B4:B55")),0)</f>
         <v>11</v>
       </c>
       <c r="D27" s="32" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C28" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D28&amp;"'!B4:B55")),0)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D28" s="32" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C29" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D29&amp;"'!B4:B55")),0)</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D29" s="32" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="C30" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D30&amp;"'!B4:B55")),0)</f>
         <v>4</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="C31" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D31&amp;"'!B4:B55")),0)</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D31" s="32" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>551</v>
-      </c>
-      <c r="B32" s="40" t="s">
-        <v>566</v>
+        <v>5</v>
+      </c>
+      <c r="B32" s="41" t="s">
+        <v>6</v>
       </c>
       <c r="C32" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D32&amp;"'!B4:B55")),0)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D32" s="32" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="C33" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D33&amp;"'!B4:B55")),0)</f>
+        <v>7</v>
+      </c>
+      <c r="D33" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="D33" s="32" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="C34" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D34&amp;"'!B4:B55")),0)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D34" s="32" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="C35" s="13">
         <f ca="1">IFERROR(COUNTA(INDIRECT("'"&amp;D35&amp;"'!B4:B55")),0)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D35" s="32" t="s">
-        <v>61</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F43" t="s">
+        <v>568</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D35" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D35">
+      <sortCondition ref="A2:A35"/>
+    </sortState>
+  </autoFilter>
+  <mergeCells count="2">
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D3" location="rol!A1" display="rol" xr:uid="{2B4614B3-B5C2-49A8-B649-B3B7A56F5F1E}"/>
-    <hyperlink ref="D4" location="usuario!A1" display="usuario" xr:uid="{EF6474E4-B295-4286-91B1-AD4657BD0CAD}"/>
-    <hyperlink ref="D5" location="usuario_rol!A1" display="usuario_rol" xr:uid="{5CADD67B-ADEE-4809-9265-387EC8F2DA1E}"/>
-    <hyperlink ref="D6" location="area!A1" display="area" xr:uid="{13DEA009-702D-4051-B272-D43DBD7A71D4}"/>
-    <hyperlink ref="D7" location="usuario_area!A1" display="usuario_area" xr:uid="{0F1E2726-E2B5-416A-B405-257D796E22CC}"/>
-    <hyperlink ref="D8" location="sistema!A1" display="sistema" xr:uid="{ADAA6A1D-4B15-4E60-9776-FCF2FC3DFD1C}"/>
-    <hyperlink ref="D9" location="area_sistema!A1" display="area_sistema" xr:uid="{795CB534-5703-4B70-B2D0-8B0E6AE13037}"/>
-    <hyperlink ref="D10" location="tipo_solicitud!A1" display="tipo_solicitud" xr:uid="{B2DB8C43-5E3D-488B-B173-D3EB88D51C09}"/>
-    <hyperlink ref="D11" location="prioridad_solicitud!A1" display="prioridad_solicitud" xr:uid="{3FA2CEDC-2839-41D0-A495-D9919BC6EBF7}"/>
-    <hyperlink ref="D12" location="estado_solicitud!A1" display="estado_solicitud" xr:uid="{1F073571-531A-4F1B-A954-5DDF15E6A1C9}"/>
-    <hyperlink ref="D13" location="solicitud!A1" display="solicitud" xr:uid="{632C16CC-3B6E-48E3-8D34-6C8DDE3803B4}"/>
-    <hyperlink ref="D14" location="'solicitud_desarrollador'!A1" display="solicitud_desarrollador" xr:uid="{74970300-8BD4-42BA-BF7C-880FC2F65753}"/>
-    <hyperlink ref="D15" location="solicitud_historial_estado!A1" display="solicitud_historial_estado" xr:uid="{242F7E10-6D13-44A7-8FA4-026C89728791}"/>
-    <hyperlink ref="D16" location="solicitud_aprobacion!A1" display="solicitud_aprobacion" xr:uid="{B093588F-7E4E-43D4-93F8-21380A0EF26D}"/>
-    <hyperlink ref="D17" location="solicitud_comentario!A1" display="solicitud_comentario" xr:uid="{D2F3E127-2BAF-49DD-9250-B1B182FB42BF}"/>
-    <hyperlink ref="D18" location="solicitud_adjunto!A1" display="solicitud_adjunto" xr:uid="{C256EC25-1819-4E94-A290-CE63736A8BBB}"/>
-    <hyperlink ref="D19" location="notificacion!A1" display="notificacion" xr:uid="{0A5FDBCB-4F45-4BFA-809C-5C86F9F68072}"/>
-    <hyperlink ref="D20" location="usuario_credencial!A1" display="usuario_credencial" xr:uid="{6DCD632A-A57E-498E-8C09-B502DF634D2D}"/>
-    <hyperlink ref="D21" location="menu_opcion!A1" display="menu_opcion" xr:uid="{4487E834-90EB-4CB1-BA2B-EF51886DFA66}"/>
-    <hyperlink ref="D22" location="rol_menu_opcion!A1" display="rol_menu_opcion" xr:uid="{DB31B0C5-ABD0-427E-ADAD-A59CF79CA713}"/>
-    <hyperlink ref="D23" location="tipo_modificacion!A1" display="tipo_modificacion" xr:uid="{2318DC5E-151D-4539-9F62-B7877DC48FA4}"/>
-    <hyperlink ref="D24" location="solicitud_modificacion!A1" display="solicitud_modificacion" xr:uid="{C47F83B0-D9FF-4067-8A85-DC81084EE9F4}"/>
-    <hyperlink ref="D25" location="solicitud_requerimiento_tecnico!A1" display="solicitud_requerimiento_tecnico" xr:uid="{026C352A-D6A5-4212-BCFB-557505736F5C}"/>
-    <hyperlink ref="D26" location="tarea_desarrollo!A1" display="tarea_desarrollo" xr:uid="{E9BD436A-F838-4EEA-9476-0D70FAB6C8A7}"/>
-    <hyperlink ref="D27" location="tarea_desarrollo_asignacion!A1" display="tarea_desarrollo_asignacion" xr:uid="{02665E46-86D7-45DC-B388-4A7F2A38E402}"/>
-    <hyperlink ref="D28" location="actividad_reciente!A1" display="actividad_reciente" xr:uid="{A28BE65C-2567-4017-9291-86D89FCD485D}"/>
-    <hyperlink ref="D29" location="proyecto!A1" display="proyecto" xr:uid="{0215288B-2E91-4CFB-B049-6FE438EEDBCF}"/>
-    <hyperlink ref="D30" location="proyecto_solicitud!A1" display="proyecto_solicitud" xr:uid="{7006D0C4-1325-443E-921A-51685992685F}"/>
-    <hyperlink ref="D31" location="proyecto_miembro!A1" display="proyecto_miembro" xr:uid="{A80B0950-37B5-4D7E-9B42-696F6382A1F2}"/>
-    <hyperlink ref="D33" location="documento_proyecto!A1" display="documento_proyecto" xr:uid="{0808F433-6682-4B84-95C8-51AC0C062DD1}"/>
-    <hyperlink ref="D35" location="evento_participante!A1" display="evento_participante" xr:uid="{70A16F5F-9B82-4A64-9262-91F18251F6DC}"/>
-    <hyperlink ref="D34" location="evento_calendario!A1" display="evento_calendario" xr:uid="{DFC53FFB-E375-46CF-9532-85DA4ADF49D7}"/>
-    <hyperlink ref="D32" location="sistema_desarrollador!A1" display="sistema_desarrollador" xr:uid="{DAB7F0B9-F482-4DA8-868D-D78D6B0583BF}"/>
+    <hyperlink ref="D16" location="rol!A1" display="rol" xr:uid="{2B4614B3-B5C2-49A8-B649-B3B7A56F5F1E}"/>
+    <hyperlink ref="D32" location="usuario!A1" display="usuario" xr:uid="{EF6474E4-B295-4286-91B1-AD4657BD0CAD}"/>
+    <hyperlink ref="D35" location="usuario_rol!A1" display="usuario_rol" xr:uid="{5CADD67B-ADEE-4809-9265-387EC8F2DA1E}"/>
+    <hyperlink ref="D4" location="area!A1" display="area" xr:uid="{13DEA009-702D-4051-B272-D43DBD7A71D4}"/>
+    <hyperlink ref="D33" location="usuario_area!A1" display="usuario_area" xr:uid="{0F1E2726-E2B5-416A-B405-257D796E22CC}"/>
+    <hyperlink ref="D18" location="sistema!A1" display="sistema" xr:uid="{ADAA6A1D-4B15-4E60-9776-FCF2FC3DFD1C}"/>
+    <hyperlink ref="D5" location="area_sistema!A1" display="area_sistema" xr:uid="{795CB534-5703-4B70-B2D0-8B0E6AE13037}"/>
+    <hyperlink ref="D31" location="tipo_solicitud!A1" display="tipo_solicitud" xr:uid="{B2DB8C43-5E3D-488B-B173-D3EB88D51C09}"/>
+    <hyperlink ref="D12" location="prioridad_solicitud!A1" display="prioridad_solicitud" xr:uid="{3FA2CEDC-2839-41D0-A495-D9919BC6EBF7}"/>
+    <hyperlink ref="D7" location="estado_solicitud!A1" display="estado_solicitud" xr:uid="{1F073571-531A-4F1B-A954-5DDF15E6A1C9}"/>
+    <hyperlink ref="D20" location="solicitud!A1" display="solicitud" xr:uid="{632C16CC-3B6E-48E3-8D34-6C8DDE3803B4}"/>
+    <hyperlink ref="D24" location="'solicitud_desarrollador'!A1" display="solicitud_desarrollador" xr:uid="{74970300-8BD4-42BA-BF7C-880FC2F65753}"/>
+    <hyperlink ref="D25" location="solicitud_historial_estado!A1" display="solicitud_historial_estado" xr:uid="{242F7E10-6D13-44A7-8FA4-026C89728791}"/>
+    <hyperlink ref="D22" location="solicitud_aprobacion!A1" display="solicitud_aprobacion" xr:uid="{B093588F-7E4E-43D4-93F8-21380A0EF26D}"/>
+    <hyperlink ref="D23" location="solicitud_comentario!A1" display="solicitud_comentario" xr:uid="{D2F3E127-2BAF-49DD-9250-B1B182FB42BF}"/>
+    <hyperlink ref="D21" location="solicitud_adjunto!A1" display="solicitud_adjunto" xr:uid="{C256EC25-1819-4E94-A290-CE63736A8BBB}"/>
+    <hyperlink ref="D11" location="notificacion!A1" display="notificacion" xr:uid="{0A5FDBCB-4F45-4BFA-809C-5C86F9F68072}"/>
+    <hyperlink ref="D34" location="usuario_credencial!A1" display="usuario_credencial" xr:uid="{6DCD632A-A57E-498E-8C09-B502DF634D2D}"/>
+    <hyperlink ref="D10" location="menu_opcion!A1" display="menu_opcion" xr:uid="{4487E834-90EB-4CB1-BA2B-EF51886DFA66}"/>
+    <hyperlink ref="D17" location="rol_menu_opcion!A1" display="rol_menu_opcion" xr:uid="{DB31B0C5-ABD0-427E-ADAD-A59CF79CA713}"/>
+    <hyperlink ref="D30" location="tipo_modificacion!A1" display="tipo_modificacion" xr:uid="{2318DC5E-151D-4539-9F62-B7877DC48FA4}"/>
+    <hyperlink ref="D26" location="solicitud_modificacion!A1" display="solicitud_modificacion" xr:uid="{C47F83B0-D9FF-4067-8A85-DC81084EE9F4}"/>
+    <hyperlink ref="D27" location="solicitud_requerimiento_tecnico!A1" display="solicitud_requerimiento_tecnico" xr:uid="{026C352A-D6A5-4212-BCFB-557505736F5C}"/>
+    <hyperlink ref="D28" location="tarea_desarrollo!A1" display="tarea_desarrollo" xr:uid="{E9BD436A-F838-4EEA-9476-0D70FAB6C8A7}"/>
+    <hyperlink ref="D29" location="tarea_desarrollo_asignacion!A1" display="tarea_desarrollo_asignacion" xr:uid="{02665E46-86D7-45DC-B388-4A7F2A38E402}"/>
+    <hyperlink ref="D3" location="actividad_reciente!A1" display="actividad_reciente" xr:uid="{A28BE65C-2567-4017-9291-86D89FCD485D}"/>
+    <hyperlink ref="D13" location="proyecto!A1" display="proyecto" xr:uid="{0215288B-2E91-4CFB-B049-6FE438EEDBCF}"/>
+    <hyperlink ref="D15" location="proyecto_solicitud!A1" display="proyecto_solicitud" xr:uid="{7006D0C4-1325-443E-921A-51685992685F}"/>
+    <hyperlink ref="D14" location="proyecto_miembro!A1" display="proyecto_miembro" xr:uid="{A80B0950-37B5-4D7E-9B42-696F6382A1F2}"/>
+    <hyperlink ref="D6" location="documento_proyecto!A1" display="documento_proyecto" xr:uid="{0808F433-6682-4B84-95C8-51AC0C062DD1}"/>
+    <hyperlink ref="D9" location="evento_participante!A1" display="evento_participante" xr:uid="{70A16F5F-9B82-4A64-9262-91F18251F6DC}"/>
+    <hyperlink ref="D8" location="evento_calendario!A1" display="evento_calendario" xr:uid="{DFC53FFB-E375-46CF-9532-85DA4ADF49D7}"/>
+    <hyperlink ref="D19" location="sistema_desarrollador!A1" display="sistema_desarrollador" xr:uid="{DAB7F0B9-F482-4DA8-868D-D78D6B0583BF}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6858,7 +6943,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
@@ -6924,7 +7009,7 @@
         <v>72</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>197</v>
+        <v>570</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>123</v>
@@ -6933,10 +7018,10 @@
         <v>107</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>71</v>
+        <v>571</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>474</v>
+        <v>572</v>
       </c>
       <c r="G4" s="4"/>
     </row>
@@ -6945,7 +7030,7 @@
         <v>94</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>122</v>
+        <v>197</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>132</v>
@@ -6955,88 +7040,92 @@
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="7" t="s">
-        <v>475</v>
+        <v>573</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>133</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
+      <c r="A6" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="B6" s="4" t="s">
-        <v>125</v>
+        <v>84</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>126</v>
+        <v>93</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>107</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="7" t="s">
-        <v>476</v>
-      </c>
-      <c r="G6" s="4"/>
+        <v>574</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
-        <v>77</v>
+        <v>575</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>138</v>
+        <v>104</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="7" t="s">
-        <v>477</v>
+        <v>576</v>
       </c>
       <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>94</v>
-      </c>
+      <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E8" s="17"/>
+      <c r="E8" s="4">
+        <v>1</v>
+      </c>
       <c r="F8" s="7" t="s">
-        <v>478</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>129</v>
-      </c>
+        <v>577</v>
+      </c>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
-        <v>198</v>
+        <v>97</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="F9" s="7" t="s">
-        <v>479</v>
+        <v>578</v>
       </c>
       <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>82</v>
@@ -7046,83 +7135,9 @@
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="7" t="s">
-        <v>480</v>
+        <v>579</v>
       </c>
       <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="7" t="s">
-        <v>481</v>
-      </c>
-      <c r="G11" s="4"/>
-    </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="7" t="s">
-        <v>482</v>
-      </c>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="7" t="s">
-        <v>483</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E14" s="4">
-        <v>1</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>484</v>
-      </c>
-      <c r="G14" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9333,7 +9348,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -9494,6 +9509,25 @@
         <v>253</v>
       </c>
       <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="G9" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10291,21 +10325,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005142CE7EA3A7964E9436DBE7E03CB6CB" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="63db46f1abc2b6b278c21e483c5aa9be">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6bcc5027-7626-4b3f-a1b8-943f1b440c70" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="76940422befb73c746558f8c0b4d7441" ns2:_="">
     <xsd:import namespace="6bcc5027-7626-4b3f-a1b8-943f1b440c70"/>
@@ -10467,10 +10486,35 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D579197-D438-4EF6-9CBD-9164EE63483F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C3E8581-B97A-4720-A878-3739A3D458F9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6bcc5027-7626-4b3f-a1b8-943f1b440c70"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10492,19 +10536,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C3E8581-B97A-4720-A878-3739A3D458F9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D579197-D438-4EF6-9CBD-9164EE63483F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6bcc5027-7626-4b3f-a1b8-943f1b440c70"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>